<commit_message>
Add Baseline/Load Testing category with 310 test cases in Python and JS frameworks
</commit_message>
<xml_diff>
--- a/Test_Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test_Results/Excel/Failed_Test_Cases.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0.097s</t>
+          <t>0.301s</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0.443s</t>
+          <t>0.207s</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.375s</t>
+          <t>0.258s</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.114s</t>
+          <t>0.119s</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">

</xml_diff>